<commit_message>
Elv: ms env e nutri completos
</commit_message>
<xml_diff>
--- a/res/tabela de nutrientes.xlsx
+++ b/res/tabela de nutrientes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/480d9b848b88e342/MSS/_Zoo-Rebio/ZooRebio3-23_24/rebio23-part/res/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="54" documentId="11_8EC6323DEB31E2B420E422BF073E1BAD2A5940E2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{03F455EC-7D20-4329-ADB7-F25B5C3C3A77}"/>
+  <xr:revisionPtr revIDLastSave="62" documentId="11_8EC6323DEB31E2B420E422BF073E1BAD2A5940E2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B7672DA9-897E-4FBD-9598-AFBAC5A4A9E4}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-22425" windowWidth="21840" windowHeight="37920" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20490" yWindow="-21510" windowWidth="19470" windowHeight="13380" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
@@ -421,7 +421,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -443,6 +443,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1065,7 +1068,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="8" t="s">
         <v>104</v>
       </c>
       <c r="C1" s="1"/>
@@ -1073,7 +1076,7 @@
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="8" t="s">
         <v>105</v>
       </c>
       <c r="I1" s="1"/>
@@ -1132,7 +1135,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>99</v>
       </c>
@@ -1182,7 +1185,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>100</v>
       </c>
@@ -1332,7 +1335,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>103</v>
       </c>
@@ -1383,10 +1386,6 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B1:G1"/>
-    <mergeCell ref="H1:P1"/>
-  </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>